<commit_message>
auto: session 2026-08-20 10:35
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/NOIBO-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
+++ b/11-bao-gia-khach/NOIBO-Booking-Bao-PR-DigicomVN-2026-08-20.xlsx
@@ -608,8 +608,6 @@
           <t>⚠ FILE NỘI BỘ - TUYỆT ĐỐI KHÔNG GỬI KHÁCH ⚠</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -720,12 +718,6 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
@@ -733,12 +725,6 @@
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -746,12 +732,6 @@
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -3097,11 +3077,6 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
@@ -3109,11 +3084,6 @@
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -3121,11 +3091,6 @@
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -3937,9 +3902,6 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
@@ -3947,9 +3909,6 @@
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -3957,9 +3916,6 @@
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -4676,11 +4632,6 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
@@ -4688,11 +4639,6 @@
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -4700,11 +4646,6 @@
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -4736,11 +4677,6 @@
           <t>Gói textlink đặt đồng loạt trên nhiều trang báo (không chọn riêng từng báo). Đơn hàng từ 2 gói trở lên được hỗ trợ chiết khấu thêm - liên hệ để biết chi tiết.</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -5290,11 +5226,6 @@
           <t>Áp dụng trên 33 trang báo (danh sách minh hoạ, có thể thay đổi theo đợt triển khai):</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="18" t="inlineStr">
@@ -5302,11 +5233,6 @@
           <t>hanoitimes.vn, thieunien.vn, thanhnienviet.vn, tapchinghiencuuphathoc.vn, www.phunuvagiadinh.vn, reatimes.vn, doanhnghiephoinhap.vn, baothainguyen.vn, huengaynay.vn, baocamau.vn, baotuyenquang.com.vn, baogialai.com.vn, nguoidothi.net.vn, baolangson.vn, baolaocai.vn, baoangiang.com.vn, baocantho.com.vn, truyenhinhnghean.vn, thuonghieucongluan.com.vn, baovanhoa.vn, tapchitoaan.vn, baodanang.vn, baodongnai.com.vn, giaoducthoidai.vn, baophapluat.vn, vnreview.vn, home.vn, congly.vn, www.anninhthudo.vn, hanoimoi.vn, thuonghieuvaphapluat.vn, anhp.vn, vietq.vn</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -5356,16 +5282,6 @@
           <t>CÔNG TY TNHH DỊCH VỤ TRUYỀN THÔNG DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
@@ -5376,16 +5292,6 @@
           <t>MST: 0109816406 | STK: 567898838 - Ngân hàng TMCP Quân đội (MB Bank) - Chủ TK: CONG TY TNHH DVTT DIGITO COMBAT</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
@@ -5396,16 +5302,6 @@
           <t>Email: sales@digicomvn.com - Hotline: 0988 769 317 | ★ MIỄN PHÍ 100% PHÍ VIẾT BÀI PR ★ | Báo giá hiệu lực đến hết 27/08/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
@@ -5517,29 +5413,18 @@
           <t>Giá Link Home</t>
         </is>
       </c>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
       <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Giá Link Chuyên mục</t>
         </is>
       </c>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
       <c r="L8" s="8" t="inlineStr">
         <is>
           <t>Giá Link Fullsite</t>
         </is>
       </c>
-      <c r="M8" s="8" t="n"/>
-      <c r="N8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
       <c r="F9" s="8" t="inlineStr">
         <is>
           <t>3 tháng</t>
@@ -7177,8 +7062,8 @@
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>